<commit_message>
feat: Add new Excel input files and update processing logic
- Introduced new Excel files for client and contract data in the input directory.
- Updated the main processing script to handle new input formats and added logic for monthly date generation with a maximum date limit.
- Enhanced detail generation functions to include a new parameter for increment month, improving flexibility in calculations.
- Implemented changes in the detail and summary builders to accommodate new data structures and ensure accurate reporting.
- Added functionality to extract and display IVA and base amounts in the output reports.
- Cleaned up code for better readability and maintainability, including renaming variables and functions for clarity.
- Removed deprecated references to the old file paths and ensured compatibility with the new directory structure.
</commit_message>
<xml_diff>
--- a/data/input/base_inpc.xlsx
+++ b/data/input/base_inpc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\amer.prgx.com\Citrix\UserHomeDir\opined01\Desktop\Automation-Subarrenda\data\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Soriana\00 - AUDITORIA 2020 - 2024\00 - Auditores\Oscar\Proyectos Python\Automation-Subarrenda\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD63DA55-156D-4A04-8644-AFA918AF7F12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5904AD95-1E7A-47B7-AFC4-64E69C491C09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{7FF57DCB-0663-4083-A355-97AE95016C18}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15840" xr2:uid="{021D5AA9-46E5-4F5F-844E-30F1C97950B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -461,14 +461,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5950A2A3-5663-48F9-8854-99D19998FB9A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{701A9A95-F170-4564-AE58-2CDE0E2D82CF}">
   <dimension ref="A1:F311"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -488,7 +488,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>36526</v>
       </c>
@@ -508,7 +508,7 @@
         <v>0.11019999999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>36557</v>
       </c>
@@ -528,7 +528,7 @@
         <v>0.1052</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>36586</v>
       </c>
@@ -548,7 +548,7 @@
         <v>0.1011</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>36617</v>
       </c>
@@ -568,7 +568,7 @@
         <v>9.7299999999999998E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>36647</v>
       </c>
@@ -588,7 +588,7 @@
         <v>9.4800000000000009E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>36678</v>
       </c>
@@ -608,7 +608,7 @@
         <v>9.4100000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>36708</v>
       </c>
@@ -628,7 +628,7 @@
         <v>9.1199999999999989E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>36739</v>
       </c>
@@ -648,7 +648,7 @@
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>36770</v>
       </c>
@@ -668,7 +668,7 @@
         <v>8.8499999999999995E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>36800</v>
       </c>
@@ -688,7 +688,7 @@
         <v>8.9099999999999999E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>36831</v>
       </c>
@@ -708,7 +708,7 @@
         <v>8.8699999999999987E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>36861</v>
       </c>
@@ -728,7 +728,7 @@
         <v>8.9600000000000013E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>36892</v>
       </c>
@@ -748,7 +748,7 @@
         <v>8.1099999999999992E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>36923</v>
       </c>
@@ -768,7 +768,7 @@
         <v>7.0900000000000005E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>36951</v>
       </c>
@@ -788,7 +788,7 @@
         <v>7.17E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>36982</v>
       </c>
@@ -808,7 +808,7 @@
         <v>7.1099999999999997E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>37012</v>
       </c>
@@ -828,7 +828,7 @@
         <v>6.9500000000000006E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>37043</v>
       </c>
@@ -848,7 +848,7 @@
         <v>6.5700000000000008E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>37073</v>
       </c>
@@ -868,7 +868,7 @@
         <v>5.8799999999999998E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>37104</v>
       </c>
@@ -888,7 +888,7 @@
         <v>5.9299999999999999E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>37135</v>
       </c>
@@ -908,7 +908,7 @@
         <v>6.1399999999999996E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>37165</v>
       </c>
@@ -928,7 +928,7 @@
         <v>5.8899999999999994E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>37196</v>
       </c>
@@ -948,7 +948,7 @@
         <v>5.3899999999999997E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>37226</v>
       </c>
@@ -968,7 +968,7 @@
         <v>4.4000000000000004E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>37257</v>
       </c>
@@ -988,7 +988,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>37288</v>
       </c>
@@ -1008,7 +1008,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>37316</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>4.6600000000000003E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>37347</v>
       </c>
@@ -1048,7 +1048,7 @@
         <v>4.7E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>37377</v>
       </c>
@@ -1068,7 +1068,7 @@
         <v>4.6799999999999994E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>37408</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>4.9400000000000006E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>37438</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>5.5099999999999996E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>37469</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>5.2900000000000003E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>37500</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>37530</v>
       </c>
@@ -1168,7 +1168,7 @@
         <v>4.9400000000000006E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>37561</v>
       </c>
@@ -1188,7 +1188,7 @@
         <v>5.3899999999999997E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>37591</v>
       </c>
@@ -1208,7 +1208,7 @@
         <v>5.7000000000000002E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37622</v>
       </c>
@@ -1228,7 +1228,7 @@
         <v>5.16E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>37653</v>
       </c>
@@ -1248,7 +1248,7 @@
         <v>5.5199999999999999E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>37681</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>5.6399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>37712</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>5.2499999999999998E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>37742</v>
       </c>
@@ -1308,7 +1308,7 @@
         <v>4.7E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>37773</v>
       </c>
@@ -1328,7 +1328,7 @@
         <v>4.2699999999999995E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>37803</v>
       </c>
@@ -1348,7 +1348,7 @@
         <v>4.1299999999999996E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>37834</v>
       </c>
@@ -1368,7 +1368,7 @@
         <v>4.0399999999999998E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>37865</v>
       </c>
@@ -1388,7 +1388,7 @@
         <v>4.0399999999999998E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>37895</v>
       </c>
@@ -1408,7 +1408,7 @@
         <v>3.9599999999999996E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>37926</v>
       </c>
@@ -1428,7 +1428,7 @@
         <v>3.9800000000000002E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>37956</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>3.9800000000000002E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>37987</v>
       </c>
@@ -1468,7 +1468,7 @@
         <v>4.2000000000000003E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>38018</v>
       </c>
@@ -1488,7 +1488,7 @@
         <v>4.53E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>38047</v>
       </c>
@@ -1508,7 +1508,7 @@
         <v>4.2300000000000004E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>38078</v>
       </c>
@@ -1528,7 +1528,7 @@
         <v>4.2099999999999999E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>38108</v>
       </c>
@@ -1548,7 +1548,7 @@
         <v>4.2900000000000001E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>38139</v>
       </c>
@@ -1568,7 +1568,7 @@
         <v>4.3700000000000003E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>38169</v>
       </c>
@@ -1588,7 +1588,7 @@
         <v>4.4900000000000002E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>38200</v>
       </c>
@@ -1608,7 +1608,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>38231</v>
       </c>
@@ -1628,7 +1628,7 @@
         <v>5.0599999999999999E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>38261</v>
       </c>
@@ -1648,7 +1648,7 @@
         <v>5.4000000000000006E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>38292</v>
       </c>
@@ -1668,7 +1668,7 @@
         <v>5.4299999999999994E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>38322</v>
       </c>
@@ -1688,7 +1688,7 @@
         <v>5.1900000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>38353</v>
       </c>
@@ -1708,7 +1708,7 @@
         <v>4.5400000000000003E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>38384</v>
       </c>
@@ -1728,7 +1728,7 @@
         <v>4.2699999999999995E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>38412</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>4.3899999999999995E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>38443</v>
       </c>
@@ -1768,7 +1768,7 @@
         <v>4.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>38473</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>4.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>38504</v>
       </c>
@@ -1808,7 +1808,7 @@
         <v>4.3299999999999998E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>38534</v>
       </c>
@@ -1828,7 +1828,7 @@
         <v>4.4699999999999997E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>38565</v>
       </c>
@@ -1848,7 +1848,7 @@
         <v>3.95E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>38596</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>3.5099999999999999E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>38626</v>
       </c>
@@ -1888,7 +1888,7 @@
         <v>3.0499999999999999E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>38657</v>
       </c>
@@ -1908,7 +1908,7 @@
         <v>2.9100000000000001E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>38687</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>3.3300000000000003E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>38718</v>
       </c>
@@ -1948,7 +1948,7 @@
         <v>3.9399999999999998E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>38749</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>38777</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>3.4099999999999998E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>38808</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>38838</v>
       </c>
@@ -2028,7 +2028,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>38869</v>
       </c>
@@ -2048,7 +2048,7 @@
         <v>3.1800000000000002E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>38899</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>3.0600000000000002E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>38930</v>
       </c>
@@ -2088,7 +2088,7 @@
         <v>3.4700000000000002E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>38961</v>
       </c>
@@ -2108,7 +2108,7 @@
         <v>4.0899999999999999E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>38991</v>
       </c>
@@ -2128,7 +2128,7 @@
         <v>4.2900000000000001E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>39022</v>
       </c>
@@ -2148,7 +2148,7 @@
         <v>4.0899999999999999E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>39052</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>4.0500000000000001E-2</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>39083</v>
       </c>
@@ -2188,7 +2188,7 @@
         <v>3.9800000000000002E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>39114</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>4.1100000000000005E-2</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>39142</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>4.2099999999999999E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>39173</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>3.9900000000000005E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>39203</v>
       </c>
@@ -2268,7 +2268,7 @@
         <v>3.95E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>39234</v>
       </c>
@@ -2288,7 +2288,7 @@
         <v>3.9800000000000002E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>39264</v>
       </c>
@@ -2308,7 +2308,7 @@
         <v>4.1399999999999999E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>39295</v>
       </c>
@@ -2328,7 +2328,7 @@
         <v>4.0300000000000002E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>39326</v>
       </c>
@@ -2348,7 +2348,7 @@
         <v>3.7900000000000003E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>39356</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>3.7400000000000003E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>39387</v>
       </c>
@@ -2388,7 +2388,7 @@
         <v>3.9300000000000002E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>39417</v>
       </c>
@@ -2408,7 +2408,7 @@
         <v>3.7599999999999995E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>39448</v>
       </c>
@@ -2428,7 +2428,7 @@
         <v>3.7000000000000005E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>39479</v>
       </c>
@@ -2448,7 +2448,7 @@
         <v>3.7200000000000004E-2</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>39508</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>4.2500000000000003E-2</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>39539</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>4.5499999999999999E-2</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>39569</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>39600</v>
       </c>
@@ -2528,7 +2528,7 @@
         <v>5.2600000000000001E-2</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>39630</v>
       </c>
@@ -2548,7 +2548,7 @@
         <v>5.3899999999999997E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>39661</v>
       </c>
@@ -2568,7 +2568,7 @@
         <v>5.57E-2</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>39692</v>
       </c>
@@ -2588,7 +2588,7 @@
         <v>5.4699999999999999E-2</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>39722</v>
       </c>
@@ -2608,7 +2608,7 @@
         <v>5.7800000000000004E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
         <v>39753</v>
       </c>
@@ -2628,7 +2628,7 @@
         <v>6.2300000000000001E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
         <v>39783</v>
       </c>
@@ -2648,7 +2648,7 @@
         <v>6.5299999999999997E-2</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
         <v>39814</v>
       </c>
@@ -2668,7 +2668,7 @@
         <v>6.2800000000000009E-2</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
         <v>39845</v>
       </c>
@@ -2688,7 +2688,7 @@
         <v>6.2E-2</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
         <v>39873</v>
       </c>
@@ -2708,7 +2708,7 @@
         <v>6.0400000000000002E-2</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
         <v>39904</v>
       </c>
@@ -2728,7 +2728,7 @@
         <v>6.1699999999999998E-2</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
         <v>39934</v>
       </c>
@@ -2748,7 +2748,7 @@
         <v>5.9800000000000006E-2</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
         <v>39965</v>
       </c>
@@ -2768,7 +2768,7 @@
         <v>5.74E-2</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
         <v>39995</v>
       </c>
@@ -2788,7 +2788,7 @@
         <v>5.4400000000000004E-2</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
         <v>40026</v>
       </c>
@@ -2808,7 +2808,7 @@
         <v>5.0799999999999998E-2</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
         <v>40057</v>
       </c>
@@ -2828,7 +2828,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
         <v>40087</v>
       </c>
@@ -2848,7 +2848,7 @@
         <v>4.4999999999999998E-2</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
         <v>40118</v>
       </c>
@@ -2868,7 +2868,7 @@
         <v>3.8599999999999995E-2</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
         <v>40148</v>
       </c>
@@ -2888,7 +2888,7 @@
         <v>3.5699999999999996E-2</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
         <v>40179</v>
       </c>
@@ -2908,7 +2908,7 @@
         <v>4.4600000000000001E-2</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
         <v>40210</v>
       </c>
@@ -2928,7 +2928,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
         <v>40238</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>4.9699999999999994E-2</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
         <v>40269</v>
       </c>
@@ -2968,7 +2968,7 @@
         <v>4.2699999999999995E-2</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
         <v>40299</v>
       </c>
@@ -2988,7 +2988,7 @@
         <v>3.9199999999999999E-2</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="1">
         <v>40330</v>
       </c>
@@ -3008,7 +3008,7 @@
         <v>3.6900000000000002E-2</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>40360</v>
       </c>
@@ -3028,7 +3028,7 @@
         <v>3.6400000000000002E-2</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
         <v>40391</v>
       </c>
@@ -3048,7 +3048,7 @@
         <v>3.6799999999999999E-2</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
         <v>40422</v>
       </c>
@@ -3068,7 +3068,7 @@
         <v>3.7000000000000005E-2</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" s="1">
         <v>40452</v>
       </c>
@@ -3088,7 +3088,7 @@
         <v>4.0199999999999993E-2</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" s="1">
         <v>40483</v>
       </c>
@@ -3108,7 +3108,7 @@
         <v>4.3200000000000002E-2</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" s="1">
         <v>40513</v>
       </c>
@@ -3128,7 +3128,7 @@
         <v>4.4000000000000004E-2</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" s="1">
         <v>40544</v>
       </c>
@@ -3148,7 +3148,7 @@
         <v>3.78E-2</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" s="1">
         <v>40575</v>
       </c>
@@ -3168,7 +3168,7 @@
         <v>3.5699999999999996E-2</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" s="1">
         <v>40603</v>
       </c>
@@ -3188,7 +3188,7 @@
         <v>3.04E-2</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="1">
         <v>40634</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>3.3599999999999998E-2</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" s="1">
         <v>40664</v>
       </c>
@@ -3228,7 +3228,7 @@
         <v>3.2500000000000001E-2</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="1">
         <v>40695</v>
       </c>
@@ -3248,7 +3248,7 @@
         <v>3.2799999999999996E-2</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" s="1">
         <v>40725</v>
       </c>
@@ -3268,7 +3268,7 @@
         <v>3.5499999999999997E-2</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" s="1">
         <v>40756</v>
       </c>
@@ -3288,7 +3288,7 @@
         <v>3.4200000000000001E-2</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" s="1">
         <v>40787</v>
       </c>
@@ -3308,7 +3308,7 @@
         <v>3.1400000000000004E-2</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" s="1">
         <v>40817</v>
       </c>
@@ -3328,7 +3328,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" s="1">
         <v>40848</v>
       </c>
@@ -3348,7 +3348,7 @@
         <v>3.4799999999999998E-2</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" s="1">
         <v>40878</v>
       </c>
@@ -3368,7 +3368,7 @@
         <v>3.8199999999999998E-2</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" s="1">
         <v>40909</v>
       </c>
@@ -3388,7 +3388,7 @@
         <v>4.0500000000000001E-2</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147" s="1">
         <v>40940</v>
       </c>
@@ -3408,7 +3408,7 @@
         <v>3.8699999999999998E-2</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" s="1">
         <v>40969</v>
       </c>
@@ -3428,7 +3428,7 @@
         <v>3.73E-2</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" s="1">
         <v>41000</v>
       </c>
@@ -3448,7 +3448,7 @@
         <v>3.4099999999999998E-2</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" s="1">
         <v>41030</v>
       </c>
@@ -3468,7 +3468,7 @@
         <v>3.85E-2</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" s="1">
         <v>41061</v>
       </c>
@@ -3488,7 +3488,7 @@
         <v>4.3400000000000001E-2</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152" s="1">
         <v>41091</v>
       </c>
@@ -3508,7 +3508,7 @@
         <v>4.4199999999999996E-2</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153" s="1">
         <v>41122</v>
       </c>
@@ -3528,7 +3528,7 @@
         <v>4.5700000000000005E-2</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" s="1">
         <v>41153</v>
       </c>
@@ -3548,7 +3548,7 @@
         <v>4.7699999999999992E-2</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" s="1">
         <v>41183</v>
       </c>
@@ -3568,7 +3568,7 @@
         <v>4.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A156" s="1">
         <v>41214</v>
       </c>
@@ -3588,7 +3588,7 @@
         <v>4.1799999999999997E-2</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157" s="1">
         <v>41244</v>
       </c>
@@ -3608,7 +3608,7 @@
         <v>3.5699999999999996E-2</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A158" s="1">
         <v>41275</v>
       </c>
@@ -3628,7 +3628,7 @@
         <v>3.2500000000000001E-2</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" s="1">
         <v>41306</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>3.5499999999999997E-2</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160" s="1">
         <v>41334</v>
       </c>
@@ -3668,7 +3668,7 @@
         <v>4.2500000000000003E-2</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="1">
         <v>41365</v>
       </c>
@@ -3688,7 +3688,7 @@
         <v>4.6500000000000007E-2</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" s="1">
         <v>41395</v>
       </c>
@@ -3708,7 +3708,7 @@
         <v>4.6300000000000001E-2</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="1">
         <v>41426</v>
       </c>
@@ -3728,7 +3728,7 @@
         <v>4.0899999999999999E-2</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" s="1">
         <v>41456</v>
       </c>
@@ -3748,7 +3748,7 @@
         <v>3.4700000000000002E-2</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" s="1">
         <v>41487</v>
       </c>
@@ -3768,7 +3768,7 @@
         <v>3.4599999999999999E-2</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" s="1">
         <v>41518</v>
       </c>
@@ -3788,7 +3788,7 @@
         <v>3.39E-2</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" s="1">
         <v>41548</v>
       </c>
@@ -3808,7 +3808,7 @@
         <v>3.3599999999999998E-2</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" s="1">
         <v>41579</v>
       </c>
@@ -3828,7 +3828,7 @@
         <v>3.6200000000000003E-2</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" s="1">
         <v>41609</v>
       </c>
@@ -3848,7 +3848,7 @@
         <v>3.9699999999999999E-2</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" s="1">
         <v>41640</v>
       </c>
@@ -3868,7 +3868,7 @@
         <v>4.4800000000000006E-2</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" s="1">
         <v>41671</v>
       </c>
@@ -3888,7 +3888,7 @@
         <v>4.2300000000000004E-2</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" s="1">
         <v>41699</v>
       </c>
@@ -3908,7 +3908,7 @@
         <v>3.7599999999999995E-2</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" s="1">
         <v>41730</v>
       </c>
@@ -3928,7 +3928,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" s="1">
         <v>41760</v>
       </c>
@@ -3948,7 +3948,7 @@
         <v>3.5099999999999999E-2</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" s="1">
         <v>41791</v>
       </c>
@@ -3968,7 +3968,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176" s="1">
         <v>41821</v>
       </c>
@@ -3988,7 +3988,7 @@
         <v>4.07E-2</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" s="1">
         <v>41852</v>
       </c>
@@ -4008,7 +4008,7 @@
         <v>4.1500000000000002E-2</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178" s="1">
         <v>41883</v>
       </c>
@@ -4028,7 +4028,7 @@
         <v>4.2199999999999994E-2</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" s="1">
         <v>41913</v>
       </c>
@@ -4048,7 +4048,7 @@
         <v>4.2999999999999997E-2</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180" s="1">
         <v>41944</v>
       </c>
@@ -4068,7 +4068,7 @@
         <v>4.1700000000000001E-2</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181" s="1">
         <v>41974</v>
       </c>
@@ -4088,7 +4088,7 @@
         <v>4.0800000000000003E-2</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182" s="1">
         <v>42005</v>
       </c>
@@ -4108,7 +4108,7 @@
         <v>3.0699999999999998E-2</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183" s="1">
         <v>42036</v>
       </c>
@@ -4128,7 +4128,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184" s="1">
         <v>42064</v>
       </c>
@@ -4148,7 +4148,7 @@
         <v>3.1400000000000004E-2</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" s="1">
         <v>42095</v>
       </c>
@@ -4168,7 +4168,7 @@
         <v>3.0600000000000002E-2</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186" s="1">
         <v>42125</v>
       </c>
@@ -4188,7 +4188,7 @@
         <v>2.8799999999999999E-2</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187" s="1">
         <v>42156</v>
       </c>
@@ -4208,7 +4208,7 @@
         <v>2.87E-2</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" s="1">
         <v>42186</v>
       </c>
@@ -4228,7 +4228,7 @@
         <v>2.7400000000000001E-2</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" s="1">
         <v>42217</v>
       </c>
@@ -4248,7 +4248,7 @@
         <v>2.5899999999999999E-2</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" s="1">
         <v>42248</v>
       </c>
@@ -4268,7 +4268,7 @@
         <v>2.52E-2</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191" s="1">
         <v>42278</v>
       </c>
@@ -4288,7 +4288,7 @@
         <v>2.4799999999999999E-2</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192" s="1">
         <v>42309</v>
       </c>
@@ -4308,7 +4308,7 @@
         <v>2.2099999999999998E-2</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193" s="1">
         <v>42339</v>
       </c>
@@ -4328,7 +4328,7 @@
         <v>2.1299999999999999E-2</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194" s="1">
         <v>42370</v>
       </c>
@@ -4348,7 +4348,7 @@
         <v>2.6099999999999998E-2</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195" s="1">
         <v>42401</v>
       </c>
@@ -4368,7 +4368,7 @@
         <v>2.87E-2</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A196" s="1">
         <v>42430</v>
       </c>
@@ -4388,7 +4388,7 @@
         <v>2.6000000000000002E-2</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A197" s="1">
         <v>42461</v>
       </c>
@@ -4408,7 +4408,7 @@
         <v>2.5399999999999999E-2</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A198" s="1">
         <v>42491</v>
       </c>
@@ -4428,7 +4428,7 @@
         <v>2.6000000000000002E-2</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A199" s="1">
         <v>42522</v>
       </c>
@@ -4448,7 +4448,7 @@
         <v>2.5399999999999999E-2</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A200" s="1">
         <v>42552</v>
       </c>
@@ -4468,7 +4468,7 @@
         <v>2.6499999999999999E-2</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A201" s="1">
         <v>42583</v>
       </c>
@@ -4488,7 +4488,7 @@
         <v>2.7300000000000001E-2</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A202" s="1">
         <v>42614</v>
       </c>
@@ -4508,7 +4508,7 @@
         <v>2.9700000000000001E-2</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A203" s="1">
         <v>42644</v>
       </c>
@@ -4528,7 +4528,7 @@
         <v>3.0600000000000002E-2</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A204" s="1">
         <v>42675</v>
       </c>
@@ -4548,7 +4548,7 @@
         <v>3.3099999999999997E-2</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" s="1">
         <v>42705</v>
       </c>
@@ -4568,7 +4568,7 @@
         <v>3.3599999999999998E-2</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A206" s="1">
         <v>42736</v>
       </c>
@@ -4588,7 +4588,7 @@
         <v>4.7199999999999999E-2</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A207" s="1">
         <v>42767</v>
       </c>
@@ -4608,7 +4608,7 @@
         <v>4.8600000000000004E-2</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A208" s="1">
         <v>42795</v>
       </c>
@@ -4628,7 +4628,7 @@
         <v>5.3499999999999999E-2</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" s="1">
         <v>42826</v>
       </c>
@@ -4648,7 +4648,7 @@
         <v>5.8200000000000002E-2</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A210" s="1">
         <v>42856</v>
       </c>
@@ -4668,7 +4668,7 @@
         <v>6.1600000000000002E-2</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A211" s="1">
         <v>42887</v>
       </c>
@@ -4688,7 +4688,7 @@
         <v>6.3099999999999989E-2</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A212" s="1">
         <v>42917</v>
       </c>
@@ -4708,7 +4708,7 @@
         <v>6.4399999999999999E-2</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A213" s="1">
         <v>42948</v>
       </c>
@@ -4728,7 +4728,7 @@
         <v>6.6600000000000006E-2</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A214" s="1">
         <v>42979</v>
       </c>
@@ -4748,7 +4748,7 @@
         <v>6.3500000000000001E-2</v>
       </c>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A215" s="1">
         <v>43009</v>
       </c>
@@ -4768,7 +4768,7 @@
         <v>6.3700000000000007E-2</v>
       </c>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A216" s="1">
         <v>43040</v>
       </c>
@@ -4788,7 +4788,7 @@
         <v>6.6299999999999998E-2</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A217" s="1">
         <v>43070</v>
       </c>
@@ -4808,7 +4808,7 @@
         <v>6.7699999999999996E-2</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A218" s="1">
         <v>43101</v>
       </c>
@@ -4828,7 +4828,7 @@
         <v>5.5500000000000001E-2</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A219" s="1">
         <v>43132</v>
       </c>
@@ -4848,7 +4848,7 @@
         <v>5.3399999999999996E-2</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A220" s="1">
         <v>43160</v>
       </c>
@@ -4868,7 +4868,7 @@
         <v>5.04E-2</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221" s="1">
         <v>43191</v>
       </c>
@@ -4888,7 +4888,7 @@
         <v>4.5499999999999999E-2</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A222" s="1">
         <v>43221</v>
       </c>
@@ -4908,7 +4908,7 @@
         <v>4.5100000000000001E-2</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A223" s="1">
         <v>43252</v>
       </c>
@@ -4928,7 +4928,7 @@
         <v>4.6500000000000007E-2</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A224" s="1">
         <v>43282</v>
       </c>
@@ -4948,7 +4948,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A225" s="1">
         <v>43313</v>
       </c>
@@ -4968,7 +4968,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A226" s="1">
         <v>43344</v>
       </c>
@@ -4988,7 +4988,7 @@
         <v>5.0199999999999995E-2</v>
       </c>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A227" s="1">
         <v>43374</v>
       </c>
@@ -5008,7 +5008,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A228" s="1">
         <v>43405</v>
       </c>
@@ -5028,7 +5028,7 @@
         <v>4.7199999999999999E-2</v>
       </c>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A229" s="1">
         <v>43435</v>
       </c>
@@ -5048,7 +5048,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A230" s="1">
         <v>43466</v>
       </c>
@@ -5068,7 +5068,7 @@
         <v>4.3700000000000003E-2</v>
       </c>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A231" s="1">
         <v>43497</v>
       </c>
@@ -5088,7 +5088,7 @@
         <v>3.9399999999999998E-2</v>
       </c>
     </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A232" s="1">
         <v>43525</v>
       </c>
@@ -5108,7 +5108,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A233" s="1">
         <v>43556</v>
       </c>
@@ -5128,7 +5128,7 @@
         <v>4.41E-2</v>
       </c>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A234" s="1">
         <v>43586</v>
       </c>
@@ -5148,7 +5148,7 @@
         <v>4.2800000000000005E-2</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A235" s="1">
         <v>43617</v>
       </c>
@@ -5168,7 +5168,7 @@
         <v>3.95E-2</v>
       </c>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A236" s="1">
         <v>43647</v>
       </c>
@@ -5188,7 +5188,7 @@
         <v>3.78E-2</v>
       </c>
     </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A237" s="1">
         <v>43678</v>
       </c>
@@ -5208,7 +5208,7 @@
         <v>3.1600000000000003E-2</v>
       </c>
     </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A238" s="1">
         <v>43709</v>
       </c>
@@ -5228,7 +5228,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A239" s="1">
         <v>43739</v>
       </c>
@@ -5248,7 +5248,7 @@
         <v>3.0200000000000001E-2</v>
       </c>
     </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A240" s="1">
         <v>43770</v>
       </c>
@@ -5268,7 +5268,7 @@
         <v>2.9700000000000001E-2</v>
       </c>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A241" s="1">
         <v>43800</v>
       </c>
@@ -5288,7 +5288,7 @@
         <v>2.8300000000000002E-2</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A242" s="1">
         <v>43831</v>
       </c>
@@ -5308,7 +5308,7 @@
         <v>3.2400000000000005E-2</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A243" s="1">
         <v>43862</v>
       </c>
@@ -5328,7 +5328,7 @@
         <v>3.7000000000000005E-2</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A244" s="1">
         <v>43891</v>
       </c>
@@ -5348,7 +5348,7 @@
         <v>3.2500000000000001E-2</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A245" s="1">
         <v>43922</v>
       </c>
@@ -5368,7 +5368,7 @@
         <v>2.1499999999999998E-2</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A246" s="1">
         <v>43952</v>
       </c>
@@ -5388,7 +5388,7 @@
         <v>2.8399999999999998E-2</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A247" s="1">
         <v>43983</v>
       </c>
@@ -5408,7 +5408,7 @@
         <v>3.3300000000000003E-2</v>
       </c>
     </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A248" s="1">
         <v>44013</v>
       </c>
@@ -5428,7 +5428,7 @@
         <v>3.6200000000000003E-2</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A249" s="1">
         <v>44044</v>
       </c>
@@ -5448,7 +5448,7 @@
         <v>4.0500000000000001E-2</v>
       </c>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A250" s="1">
         <v>44075</v>
       </c>
@@ -5468,7 +5468,7 @@
         <v>4.0099999999999997E-2</v>
       </c>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A251" s="1">
         <v>44105</v>
       </c>
@@ -5488,7 +5488,7 @@
         <v>4.0899999999999999E-2</v>
       </c>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A252" s="1">
         <v>44136</v>
       </c>
@@ -5508,7 +5508,7 @@
         <v>3.3300000000000003E-2</v>
       </c>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A253" s="1">
         <v>44166</v>
       </c>
@@ -5528,7 +5528,7 @@
         <v>3.15E-2</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A254" s="1">
         <v>44197</v>
       </c>
@@ -5548,7 +5548,7 @@
         <v>3.5400000000000001E-2</v>
       </c>
     </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A255" s="1">
         <v>44228</v>
       </c>
@@ -5568,7 +5568,7 @@
         <v>3.7599999999999995E-2</v>
       </c>
     </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A256" s="1">
         <v>44256</v>
       </c>
@@ -5588,7 +5588,7 @@
         <v>4.6699999999999998E-2</v>
       </c>
     </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A257" s="1">
         <v>44287</v>
       </c>
@@ -5608,7 +5608,7 @@
         <v>6.08E-2</v>
       </c>
     </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A258" s="1">
         <v>44317</v>
       </c>
@@ -5628,7 +5628,7 @@
         <v>5.8899999999999994E-2</v>
       </c>
     </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A259" s="1">
         <v>44348</v>
       </c>
@@ -5648,7 +5648,7 @@
         <v>5.8799999999999998E-2</v>
       </c>
     </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A260" s="1">
         <v>44378</v>
       </c>
@@ -5668,7 +5668,7 @@
         <v>5.8099999999999999E-2</v>
       </c>
     </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A261" s="1">
         <v>44409</v>
       </c>
@@ -5688,7 +5688,7 @@
         <v>5.5899999999999998E-2</v>
       </c>
     </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A262" s="1">
         <v>44440</v>
       </c>
@@ -5708,7 +5708,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A263" s="1">
         <v>44470</v>
       </c>
@@ -5728,7 +5728,7 @@
         <v>6.2400000000000004E-2</v>
       </c>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A264" s="1">
         <v>44501</v>
       </c>
@@ -5748,7 +5748,7 @@
         <v>7.3700000000000002E-2</v>
       </c>
     </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A265" s="1">
         <v>44531</v>
       </c>
@@ -5768,7 +5768,7 @@
         <v>7.3599999999999999E-2</v>
       </c>
     </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A266" s="1">
         <v>44562</v>
       </c>
@@ -5788,7 +5788,7 @@
         <v>7.0699999999999999E-2</v>
       </c>
     </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A267" s="1">
         <v>44593</v>
       </c>
@@ -5808,7 +5808,7 @@
         <v>7.2800000000000004E-2</v>
       </c>
     </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A268" s="1">
         <v>44621</v>
       </c>
@@ -5828,7 +5828,7 @@
         <v>7.4499999999999997E-2</v>
       </c>
     </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A269" s="1">
         <v>44652</v>
       </c>
@@ -5848,7 +5848,7 @@
         <v>7.6799999999999993E-2</v>
       </c>
     </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A270" s="1">
         <v>44682</v>
       </c>
@@ -5868,7 +5868,7 @@
         <v>7.6499999999999999E-2</v>
       </c>
     </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A271" s="1">
         <v>44713</v>
       </c>
@@ -5888,7 +5888,7 @@
         <v>7.9899999999999999E-2</v>
       </c>
     </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A272" s="1">
         <v>44743</v>
       </c>
@@ -5908,7 +5908,7 @@
         <v>8.1500000000000003E-2</v>
       </c>
     </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A273" s="1">
         <v>44774</v>
       </c>
@@ -5928,7 +5928,7 @@
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A274" s="1">
         <v>44805</v>
       </c>
@@ -5948,7 +5948,7 @@
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="275" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A275" s="1">
         <v>44835</v>
       </c>
@@ -5968,7 +5968,7 @@
         <v>8.4100000000000008E-2</v>
       </c>
     </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A276" s="1">
         <v>44866</v>
       </c>
@@ -5988,7 +5988,7 @@
         <v>7.8E-2</v>
       </c>
     </row>
-    <row r="277" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A277" s="1">
         <v>44896</v>
       </c>
@@ -6008,7 +6008,7 @@
         <v>7.8200000000000006E-2</v>
       </c>
     </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A278" s="1">
         <v>44927</v>
       </c>
@@ -6028,7 +6028,7 @@
         <v>7.9100000000000004E-2</v>
       </c>
     </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A279" s="1">
         <v>44958</v>
       </c>
@@ -6048,7 +6048,7 @@
         <v>7.6200000000000004E-2</v>
       </c>
     </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A280" s="1">
         <v>44986</v>
       </c>
@@ -6068,7 +6068,7 @@
         <v>6.8499999999999991E-2</v>
       </c>
     </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A281" s="1">
         <v>45017</v>
       </c>
@@ -6088,7 +6088,7 @@
         <v>6.25E-2</v>
       </c>
     </row>
-    <row r="282" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A282" s="1">
         <v>45047</v>
       </c>
@@ -6108,7 +6108,7 @@
         <v>5.8400000000000001E-2</v>
       </c>
     </row>
-    <row r="283" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A283" s="1">
         <v>45078</v>
       </c>
@@ -6128,7 +6128,7 @@
         <v>5.0599999999999999E-2</v>
       </c>
     </row>
-    <row r="284" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A284" s="1">
         <v>45108</v>
       </c>
@@ -6148,7 +6148,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="285" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A285" s="1">
         <v>45139</v>
       </c>
@@ -6168,7 +6168,7 @@
         <v>4.6399999999999997E-2</v>
       </c>
     </row>
-    <row r="286" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A286" s="1">
         <v>45170</v>
       </c>
@@ -6188,7 +6188,7 @@
         <v>4.4500000000000005E-2</v>
       </c>
     </row>
-    <row r="287" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A287" s="1">
         <v>45200</v>
       </c>
@@ -6208,7 +6208,7 @@
         <v>4.2599999999999999E-2</v>
       </c>
     </row>
-    <row r="288" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A288" s="1">
         <v>45231</v>
       </c>
@@ -6228,7 +6228,7 @@
         <v>4.3200000000000002E-2</v>
       </c>
     </row>
-    <row r="289" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A289" s="1">
         <v>45261</v>
       </c>
@@ -6248,7 +6248,7 @@
         <v>4.6600000000000003E-2</v>
       </c>
     </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A290" s="1">
         <v>45292</v>
       </c>
@@ -6268,7 +6268,7 @@
         <v>4.8799999999999996E-2</v>
       </c>
     </row>
-    <row r="291" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A291" s="1">
         <v>45323</v>
       </c>
@@ -6288,7 +6288,7 @@
         <v>4.4000000000000004E-2</v>
       </c>
     </row>
-    <row r="292" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A292" s="1">
         <v>45352</v>
       </c>
@@ -6308,7 +6308,7 @@
         <v>4.4199999999999996E-2</v>
       </c>
     </row>
-    <row r="293" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A293" s="1">
         <v>45383</v>
       </c>
@@ -6328,7 +6328,7 @@
         <v>4.6500000000000007E-2</v>
       </c>
     </row>
-    <row r="294" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A294" s="1">
         <v>45413</v>
       </c>
@@ -6348,7 +6348,7 @@
         <v>4.6900000000000004E-2</v>
       </c>
     </row>
-    <row r="295" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A295" s="1">
         <v>45444</v>
       </c>
@@ -6368,7 +6368,7 @@
         <v>4.9800000000000004E-2</v>
       </c>
     </row>
-    <row r="296" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A296" s="1">
         <v>45474</v>
       </c>
@@ -6388,7 +6388,7 @@
         <v>5.57E-2</v>
       </c>
     </row>
-    <row r="297" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A297" s="1">
         <v>45505</v>
       </c>
@@ -6408,7 +6408,7 @@
         <v>4.99E-2</v>
       </c>
     </row>
-    <row r="298" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A298" s="1">
         <v>45536</v>
       </c>
@@ -6428,7 +6428,7 @@
         <v>4.58E-2</v>
       </c>
     </row>
-    <row r="299" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A299" s="1">
         <v>45566</v>
       </c>
@@ -6448,7 +6448,7 @@
         <v>4.7599999999999996E-2</v>
       </c>
     </row>
-    <row r="300" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A300" s="1">
         <v>45597</v>
       </c>
@@ -6468,7 +6468,7 @@
         <v>4.5499999999999999E-2</v>
       </c>
     </row>
-    <row r="301" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A301" s="1">
         <v>45627</v>
       </c>
@@ -6488,7 +6488,7 @@
         <v>4.2099999999999999E-2</v>
       </c>
     </row>
-    <row r="302" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A302" s="1">
         <v>45658</v>
       </c>
@@ -6508,7 +6508,7 @@
         <v>3.5900000000000001E-2</v>
       </c>
     </row>
-    <row r="303" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A303" s="1">
         <v>45689</v>
       </c>
@@ -6528,7 +6528,7 @@
         <v>3.7699999999999997E-2</v>
       </c>
     </row>
-    <row r="304" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A304" s="1">
         <v>45717</v>
       </c>
@@ -6548,7 +6548,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="305" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A305" s="1">
         <v>45748</v>
       </c>
@@ -6568,7 +6568,7 @@
         <v>3.9300000000000002E-2</v>
       </c>
     </row>
-    <row r="306" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A306" s="1">
         <v>45778</v>
       </c>
@@ -6588,7 +6588,7 @@
         <v>4.4199999999999996E-2</v>
       </c>
     </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A307" s="1">
         <v>45809</v>
       </c>
@@ -6608,7 +6608,7 @@
         <v>4.3200000000000002E-2</v>
       </c>
     </row>
-    <row r="308" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A308" s="1">
         <v>45839</v>
       </c>
@@ -6628,7 +6628,7 @@
         <v>3.5099999999999999E-2</v>
       </c>
     </row>
-    <row r="309" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A309" s="1">
         <v>45870</v>
       </c>
@@ -6648,7 +6648,7 @@
         <v>3.5699999999999996E-2</v>
       </c>
     </row>
-    <row r="310" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A310" s="1">
         <v>45901</v>
       </c>
@@ -6668,7 +6668,7 @@
         <v>3.7599999999999995E-2</v>
       </c>
     </row>
-    <row r="311" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A311" s="1">
         <v>45931</v>
       </c>

</xml_diff>